<commit_message>
Created a master dataset with raw countries data
</commit_message>
<xml_diff>
--- a/raw data/HMBD_InputData_Metadata_06.10.2022/HMBD_InputData_Metadata_06.10.2022/AUS_InputData_27.06.2022.xlsx
+++ b/raw data/HMBD_InputData_Metadata_06.10.2022/HMBD_InputData_Metadata_06.10.2022/AUS_InputData_27.06.2022.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr showInkAnnotation="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PROJET JUMEAUX INED-MNHM\DATABASE\RAW DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ontariogov-my.sharepoint.com/personal/thiemi_doi_ontario_ca/Documents/Documents/GitHub/TwinToTwin/raw data/HMBD_InputData_Metadata_06.10.2022/HMBD_InputData_Metadata_06.10.2022/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_84E890FB34D3C8855C4BD3326856BC165B14368E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77B2734E-60DB-40AD-B140-999D42F97A72}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19430" windowHeight="10430"/>
+    <workbookView xWindow="-110" yWindow="970" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="contents" sheetId="3" r:id="rId1"/>
@@ -20,16 +21,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'input data'!$A$1:$Q$75</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -242,7 +233,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -580,34 +571,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="38">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -617,27 +607,27 @@
     <xf numFmtId="0" fontId="16" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -646,19 +636,19 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -691,7 +681,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 1"/>
+        <xdr:cNvPr id="2" name="Image 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -740,7 +736,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 2"/>
+        <xdr:cNvPr id="3" name="Image 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000003000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -969,97 +971,97 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A8:K22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="11.54296875" style="11"/>
+    <col min="1" max="16384" width="11.54296875" style="10"/>
   </cols>
   <sheetData>
     <row r="8" spans="1:4" ht="18" x14ac:dyDescent="0.4">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="14" x14ac:dyDescent="0.3">
-      <c r="A9" s="23" t="s">
+      <c r="A9" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="23" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="14" x14ac:dyDescent="0.3">
-      <c r="A10" s="23"/>
-      <c r="D10" s="24"/>
+      <c r="A10" s="22"/>
+      <c r="D10" s="23"/>
     </row>
     <row r="11" spans="1:4" ht="14" x14ac:dyDescent="0.3">
-      <c r="A11" s="23"/>
-      <c r="D11" s="24"/>
+      <c r="A11" s="22"/>
+      <c r="D11" s="23"/>
     </row>
     <row r="12" spans="1:4" ht="14" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="11" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="14" x14ac:dyDescent="0.3">
-      <c r="A13" s="9"/>
+      <c r="A13" s="8"/>
     </row>
     <row r="14" spans="1:4" ht="14" x14ac:dyDescent="0.3">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="12" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="14" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="14" x14ac:dyDescent="0.3">
-      <c r="A16" s="9"/>
+      <c r="A16" s="8"/>
     </row>
     <row r="17" spans="1:11" ht="14" x14ac:dyDescent="0.3">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="23" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="14" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="14" x14ac:dyDescent="0.3">
-      <c r="A19" s="9"/>
+      <c r="A19" s="8"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="34" t="s">
+      <c r="A20" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="B20" s="35"/>
-      <c r="C20" s="36"/>
-      <c r="D20" s="36"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="36"/>
-      <c r="J20" s="36"/>
-      <c r="K20" s="36"/>
+      <c r="B20" s="34"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="35"/>
+      <c r="E20" s="35"/>
+      <c r="F20" s="35"/>
+      <c r="G20" s="35"/>
+      <c r="H20" s="35"/>
+      <c r="I20" s="35"/>
+      <c r="J20" s="35"/>
+      <c r="K20" s="35"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="36" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:11" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A22" s="10"/>
+      <c r="A22" s="9"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A14" location="'input data'!A1" display="input data"/>
-    <hyperlink ref="A17" location="'variables input data'!A1" display="variables input data"/>
-    <hyperlink ref="D9" r:id="rId1"/>
-    <hyperlink ref="A21" r:id="rId2"/>
+    <hyperlink ref="A14" location="'input data'!A1" display="input data" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="A17" location="'variables input data'!A1" display="variables input data" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D9" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="A21" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId3"/>
@@ -1067,20 +1069,21 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:W975"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="14.453125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="14.453125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="11" style="3" customWidth="1"/>
     <col min="3" max="3" width="7.453125" style="3" customWidth="1"/>
     <col min="4" max="4" width="11" style="3" customWidth="1"/>
-    <col min="5" max="15" width="11.54296875" style="3" customWidth="1"/>
-    <col min="16" max="17" width="11" style="3" customWidth="1"/>
+    <col min="5" max="14" width="11.54296875" style="3" customWidth="1"/>
+    <col min="15" max="15" width="11.26953125" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11" style="3" customWidth="1"/>
     <col min="18" max="18" width="12.7265625" style="2" customWidth="1"/>
-    <col min="19" max="16384" width="14.453125" style="7"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="5" customFormat="1" ht="39.65" customHeight="1" x14ac:dyDescent="0.3">
@@ -1135,7 +1138,7 @@
       <c r="Q1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="33" t="s">
+      <c r="R1" s="32" t="s">
         <v>56</v>
       </c>
     </row>
@@ -2856,7 +2859,7 @@
       <c r="L32" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M32" s="8" t="s">
+      <c r="M32" s="7" t="s">
         <v>11</v>
       </c>
       <c r="N32" s="3">
@@ -7730,7 +7733,7 @@
       <c r="F114" s="3">
         <v>4446</v>
       </c>
-      <c r="G114" s="8" t="s">
+      <c r="G114" s="7" t="s">
         <v>11</v>
       </c>
       <c r="H114" s="3">
@@ -7748,7 +7751,7 @@
       <c r="L114" s="3">
         <v>4501</v>
       </c>
-      <c r="M114" s="8" t="s">
+      <c r="M114" s="7" t="s">
         <v>11</v>
       </c>
       <c r="N114" s="3">
@@ -7791,37 +7794,37 @@
       <c r="F115" s="3">
         <v>4148</v>
       </c>
-      <c r="G115" s="8" t="s">
+      <c r="G115" s="7" t="s">
         <v>11</v>
       </c>
       <c r="H115" s="3">
         <v>54</v>
       </c>
-      <c r="I115" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="J115" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="K115" s="8" t="s">
+      <c r="I115" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J115" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="K115" s="7" t="s">
         <v>11</v>
       </c>
       <c r="L115" s="3">
         <v>4202</v>
       </c>
-      <c r="M115" s="8" t="s">
+      <c r="M115" s="7" t="s">
         <v>11</v>
       </c>
       <c r="N115" s="3">
         <v>290272</v>
       </c>
-      <c r="O115" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="P115" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="Q115" s="8" t="s">
+      <c r="O115" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="P115" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q115" s="7" t="s">
         <v>11</v>
       </c>
       <c r="R115" s="2">
@@ -8694,7 +8697,7 @@
     <row r="974" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="975" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <sortState ref="A2:P113">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P113">
     <sortCondition ref="A2:A113"/>
     <sortCondition ref="C2:C113"/>
     <sortCondition ref="B2:B113"/>
@@ -8705,240 +8708,246 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B34"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.54296875" defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.90625" style="22" customWidth="1"/>
-    <col min="2" max="2" width="101.90625" style="11" customWidth="1"/>
-    <col min="3" max="16384" width="11.54296875" style="11"/>
+    <col min="1" max="1" width="29.90625" style="21" customWidth="1"/>
+    <col min="2" max="2" width="101.90625" style="10" customWidth="1"/>
+    <col min="3" max="16384" width="11.54296875" style="10"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="11"/>
+      <c r="A1" s="10"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
+      <c r="A2" s="10"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="11"/>
+      <c r="A3" s="10"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="11"/>
+      <c r="A4" s="10"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="11"/>
-      <c r="B5" s="25" t="s">
+      <c r="A5" s="10"/>
+      <c r="B5" s="24" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="11"/>
+      <c r="A6" s="10"/>
     </row>
     <row r="7" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="14"/>
+      <c r="A8" s="13"/>
     </row>
     <row r="9" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="15" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="17" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="B11" s="17" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
-        <v>2</v>
-      </c>
-      <c r="B12" s="26" t="s">
+      <c r="A12" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B12" s="25" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="38" t="s">
+      <c r="A13" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="25" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="38"/>
-      <c r="B14" s="27" t="s">
+      <c r="A14" s="37"/>
+      <c r="B14" s="26" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="38"/>
-      <c r="B15" s="27" t="s">
+      <c r="A15" s="37"/>
+      <c r="B15" s="26" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="38"/>
-      <c r="B16" s="27" t="s">
+      <c r="A16" s="37"/>
+      <c r="B16" s="26" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="38"/>
-      <c r="B17" s="28" t="s">
+      <c r="A17" s="37"/>
+      <c r="B17" s="27" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="27" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="B19" s="17" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="B20" s="17" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="B21" s="17" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="17" t="s">
+      <c r="A22" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="B22" s="17" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="17" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="17" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="17" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="20" t="s">
+      <c r="B26" s="19" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="17" t="s">
+      <c r="A27" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="17" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="17" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B29" s="20" t="s">
+      <c r="B29" s="19" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="28" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="31" t="s">
+      <c r="A31" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="31" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="30"/>
-      <c r="B32" s="30"/>
+      <c r="A32" s="29"/>
+      <c r="B32" s="29"/>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="30"/>
-      <c r="B33" s="30"/>
+      <c r="A33" s="29"/>
+      <c r="B33" s="29"/>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="21"/>
-      <c r="B34" s="21"/>
+      <c r="A34" s="20"/>
+      <c r="B34" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A13:A17"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId1"/>
+    <hyperlink ref="B5" r:id="rId1" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{034a106e-6316-442c-ad35-738afd673d2b}" enabled="1" method="Standard" siteId="{cddc1229-ac2a-4b97-b78a-0e5cacb5865c}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>